<commit_message>
Xadra v1.2: HVAC tahlili — 2 ta 96-ka (96 000 BTU/soat ≈ 56 kW) bo'yicha: sovutish 4 ssenariyda; xarajatlarda konditsioner nomi
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0121VSEFiRNp3h6KMycRzKQh
</commit_message>
<xml_diff>
--- a/xadra-filiali/hisob/Xadra_xarajatlar_v1.2.xlsx
+++ b/xadra-filiali/hisob/Xadra_xarajatlar_v1.2.xlsx
@@ -541,10 +541,10 @@
     <t xml:space="preserve">Kanalizatsiya quvuri (40 m) va otvodlar</t>
   </si>
   <si>
-    <t xml:space="preserve">Konditsioner — 2-qavat (2 ta, 100 mingtalik, o'rnatish bilan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buyurtmachi: 2 ta uchun jami, o'rnatish bilan</t>
+    <t xml:space="preserve">Konditsioner — 2-qavat (2 ta «96-ka», 96 000 BTU/soat ≈ 28 kW, o'rnatish bilan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buyurtmachi: 2 ta uchun jami, o'rnatish bilan; «100-lik» = 96-ka (09.10)</t>
   </si>
   <si>
     <t xml:space="preserve">Havo kanallari (vozduxovod), 200 m²</t>
@@ -739,7 +739,7 @@
     <t xml:space="preserve">• 3-qavat: 5-xona — o'quv xonasi (24 o'rin, bambuk panel va interaktiv doska); 2-xona — erkaklar hojatxonasi. Santexnika soni ikkala hojatxona uchun jami (2-qavatdagisi — ayollar: 2 kabina, unitazli, eng ichkarida; oldida rakovinali tambur — 6-xona 3-qavatga o'tish yo'lagi bo'lgani uchun ikki eshik orqali kiriladi); kafel faqat erkaklar hojatxonasi uchun (devor 58 m², pol 16 m²).</t>
   </si>
   <si>
-    <t xml:space="preserve">• Konditsioner va ventilyatsiya (buyurtmachi summalari, o'rnatish bilan): 2-qavatga 2 ta 100 mingtalik konditsioner va 200 m² havo kanali — «Butun qavat» qatorida; 3-qavat o'quv xonasiga 1 ta konditsioner.</t>
+    <t xml:space="preserve">• Konditsioner va ventilyatsiya (buyurtmachi summalari, o'rnatish bilan): 2-qavatga 2 ta «96-ka» (96 000 BTU/soat) konditsioner va 200 m² havo kanali — «Butun qavat» qatorida; 3-qavat o'quv xonasiga 1 ta konditsioner.</t>
   </si>
   <si>
     <t xml:space="preserve">• Santexnika: 4 ta kabina, issiq va sovuq suv quvurlari (40 m dan), 100 ta aksessuar, kanalizatsiya quvuri va otvodlar — «Hojatxonalar» qatorida.</t>
@@ -1180,7 +1180,7 @@
     <t xml:space="preserve">Qurilish chiqindisini olib chiqish (jami)</t>
   </si>
   <si>
-    <t xml:space="preserve">Konditsioner — 2 ta, 100 mingtalik, o'rnatish bilan (jami)</t>
+    <t xml:space="preserve">Konditsioner — 2 ta «96-ka» (96 000 BTU/soat), o'rnatish bilan (jami)</t>
   </si>
   <si>
     <t xml:space="preserve">Havo kanallari (vozduxovod), 200 m² (jami)</t>

</xml_diff>

<commit_message>
Konditsioner: 4-xonaga ikkala blokdan bittadan diffuzor — D7 KK1 dan (K1), D8 KK2 dan (K2)
- vent-chizma: 4-xona ikkala guruhda yarmi bilan (yuk va odam), tarmoqlar 250×150 o'z koridori magistralidan;
  6-kesishuv (D8 tarmog'i × KK2 tashqi havo kanali); KK1 35.5 kW, KK2 38.2 kW; 4-xona 910 m³/soat, CO2 ~1 670
- izoh, taqdimot: 4-xona KK1 + KK2; xarajatlar (kanal 167 m), albom qayta yig'ildi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0121VSEFiRNp3h6KMycRzKQh
</commit_message>
<xml_diff>
--- a/xadra-filiali/hisob/Xadra_xarajatlar_v1.2.xlsx
+++ b/xadra-filiali/hisob/Xadra_xarajatlar_v1.2.xlsx
@@ -1061,7 +1061,7 @@
     <t xml:space="preserve">Havo kanallari uzunligi</t>
   </si>
   <si>
-    <t xml:space="preserve">Kanallar rejasidan: 165 m (berish ~72, tashqi havo ~24, vitechka ~69) + 10% burilish va ulanishlar</t>
+    <t xml:space="preserve">Kanallar rejasidan: 167 m (berish ~75, tashqi havo ~24, vitechka ~69) + 10% burilish va ulanishlar</t>
   </si>
   <si>
     <t xml:space="preserve">TAXMIN</t>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="E6" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C6/$C$23)</f>
-        <v>0.0971685938246814</v>
+        <v>0.0971071369793098</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="E7" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C7/$C$23)</f>
-        <v>0.0458501455866683</v>
+        <v>0.0458211464502532</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="E8" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C8/$C$23)</f>
-        <v>0.104082077299537</v>
+        <v>0.104016247838816</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="E9" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C9/$C$23)</f>
-        <v>0.103629764006662</v>
+        <v>0.103564220623437</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="E10" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C10/$C$23)</f>
-        <v>0.0291534023597229</v>
+        <v>0.0291349635198637</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="E11" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C11/$C$23)</f>
-        <v>0.0379574135605796</v>
+        <v>0.0379334063911426</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2716,7 +2716,7 @@
       </c>
       <c r="E12" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C12/$C$23)</f>
-        <v>0.0265978040128532</v>
+        <v>0.026580981528714</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2736,7 +2736,7 @@
       </c>
       <c r="E13" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C13/$C$23)</f>
-        <v>0.0407941779338239</v>
+        <v>0.0407683765777822</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="E14" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C14/$C$23)</f>
-        <v>0.0067506849069547</v>
+        <v>0.00674641525786183</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2776,7 +2776,7 @@
       </c>
       <c r="E15" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C15/$C$23)</f>
-        <v>0.0189863013008101</v>
+        <v>0.0189742929127364</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2796,7 +2796,7 @@
       </c>
       <c r="E16" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C16/$C$23)</f>
-        <v>0.00427455477897405</v>
+        <v>0.00427185122382579</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2816,7 +2816,7 @@
       </c>
       <c r="E17" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C17/$C$23)</f>
-        <v>0.0416432875197768</v>
+        <v>0.0416169491219352</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2836,7 +2836,7 @@
       </c>
       <c r="E18" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C18/$C$23)</f>
-        <v>0.0156109588473327</v>
+        <v>0.0156010852838055</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2848,15 +2848,15 @@
       </c>
       <c r="C19" s="7" t="n">
         <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$345,'Hisob (batafsil)'!$C$5:$C$345,"Konditsioner va ventilyatsiya")</f>
-        <v>18238.2352941176</v>
+        <v>18288.6554621849</v>
       </c>
       <c r="D19" s="8" t="n">
         <f aca="false">C19*Narxlar!$C$19</f>
-        <v>217035000</v>
+        <v>217635000</v>
       </c>
       <c r="E19" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C19/$C$23)</f>
-        <v>0.228927327934518</v>
+        <v>0.229415013225744</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="E20" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C20/$C$23)</f>
-        <v>0.164431917210183</v>
+        <v>0.164327917898138</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2896,7 +2896,7 @@
       </c>
       <c r="E21" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C21/$C$23)</f>
-        <v>0.00464426025708149</v>
+        <v>0.00464132287193213</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="E22" s="9" t="n">
         <f aca="false">IF($C$23=0,0,C22/$C$23)</f>
-        <v>0.0294973286598419</v>
+        <v>0.0294786722947041</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2926,11 +2926,11 @@
       </c>
       <c r="C23" s="12" t="n">
         <f aca="false">SUM(C6:C22)</f>
-        <v>79668.2312184874</v>
+        <v>79718.6513865546</v>
       </c>
       <c r="D23" s="13" t="n">
         <f aca="false">C23*Narxlar!$C$19</f>
-        <v>948051951.5</v>
+        <v>948651951.5</v>
       </c>
       <c r="E23" s="14" t="n">
         <f aca="false">SUM(E6:E22)</f>
@@ -2945,11 +2945,11 @@
       </c>
       <c r="C24" s="17" t="n">
         <f aca="false">C23*Narxlar!$C$93</f>
-        <v>7966.82312184874</v>
+        <v>7971.86513865546</v>
       </c>
       <c r="D24" s="18" t="n">
         <f aca="false">C24*Narxlar!$C$19</f>
-        <v>94805195.15</v>
+        <v>94865195.15</v>
       </c>
       <c r="E24" s="16"/>
     </row>
@@ -2960,11 +2960,11 @@
       </c>
       <c r="C25" s="21" t="n">
         <f aca="false">C23+C24</f>
-        <v>87635.0543403361</v>
+        <v>87690.5165252101</v>
       </c>
       <c r="D25" s="22" t="n">
         <f aca="false">C25*Narxlar!$C$19</f>
-        <v>1042857146.65</v>
+        <v>1043517146.65</v>
       </c>
       <c r="E25" s="20"/>
     </row>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="E30" s="9" t="n">
         <f aca="false">IF($C$35=0,0,C30/$C$35)</f>
-        <v>0.0430535477886203</v>
+        <v>0.0430263174343979</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3042,7 +3042,7 @@
       </c>
       <c r="E31" s="9" t="n">
         <f aca="false">IF($C$35=0,0,C31/$C$35)</f>
-        <v>0.267071951699896</v>
+        <v>0.266903034985218</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3062,7 +3062,7 @@
       </c>
       <c r="E32" s="9" t="n">
         <f aca="false">IF($C$35=0,0,C32/$C$35)</f>
-        <v>0.135269791172409</v>
+        <v>0.135184236217744</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3074,15 +3074,15 @@
       </c>
       <c r="C33" s="7" t="n">
         <f aca="false">'Xonalar bo''yicha'!$X$36</f>
-        <v>36864.7016806723</v>
+        <v>36915.1218487395</v>
       </c>
       <c r="D33" s="8" t="n">
         <f aca="false">C33*Narxlar!$C$19</f>
-        <v>438689950</v>
+        <v>439289950</v>
       </c>
       <c r="E33" s="9" t="n">
         <f aca="false">IF($C$35=0,0,C33/$C$35)</f>
-        <v>0.462727753796518</v>
+        <v>0.463067565828963</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="E34" s="9" t="n">
         <f aca="false">IF($C$35=0,0,C34/$C$35)</f>
-        <v>0.0918769555425571</v>
+        <v>0.0918188455336773</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3112,11 +3112,11 @@
       </c>
       <c r="C35" s="12" t="n">
         <f aca="false">SUM(C30:C34)</f>
-        <v>79668.2312184874</v>
+        <v>79718.6513865546</v>
       </c>
       <c r="D35" s="13" t="n">
         <f aca="false">C35*Narxlar!$C$19</f>
-        <v>948051951.5</v>
+        <v>948651951.5</v>
       </c>
       <c r="E35" s="14" t="n">
         <f aca="false">SUM(E30:E34)</f>
@@ -3291,7 +3291,7 @@
       </c>
       <c r="K9" s="39" t="n">
         <f aca="false">IF($I$15=0,0,I9/$I$15)</f>
-        <v>0.132047615958101</v>
+        <v>0.131964098953314</v>
       </c>
       <c r="L9" s="37" t="n">
         <f aca="false">SUM($I$9:I9)</f>
@@ -3337,7 +3337,7 @@
       </c>
       <c r="K10" s="39" t="n">
         <f aca="false">IF($I$15=0,0,I10/$I$15)</f>
-        <v>0.00427455477897405</v>
+        <v>0.00427185122382579</v>
       </c>
       <c r="L10" s="37" t="n">
         <f aca="false">SUM($I$9:I10)</f>
@@ -3367,27 +3367,27 @@
       </c>
       <c r="G11" s="36" t="n">
         <f aca="false">N107</f>
-        <v>14747.4672268908</v>
+        <v>14797.887394958</v>
       </c>
       <c r="H11" s="37" t="n">
         <f aca="false">G11*Narxlar!$C$93</f>
-        <v>1474.74672268908</v>
+        <v>1479.7887394958</v>
       </c>
       <c r="I11" s="37" t="n">
         <f aca="false">G11+H11</f>
-        <v>16222.2139495798</v>
+        <v>16277.6761344538</v>
       </c>
       <c r="J11" s="38" t="n">
         <f aca="false">I11*Narxlar!$C$19</f>
-        <v>193044346</v>
+        <v>193704346</v>
       </c>
       <c r="K11" s="39" t="n">
         <f aca="false">IF($I$15=0,0,I11/$I$15)</f>
-        <v>0.185111016039083</v>
+        <v>0.18562641411485</v>
       </c>
       <c r="L11" s="37" t="n">
         <f aca="false">SUM($I$9:I11)</f>
-        <v>28168.814789916</v>
+        <v>28224.2769747899</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3429,11 +3429,11 @@
       </c>
       <c r="K12" s="39" t="n">
         <f aca="false">IF($I$15=0,0,I12/$I$15)</f>
-        <v>0.211285693450735</v>
+        <v>0.211152060229541</v>
       </c>
       <c r="L12" s="37" t="n">
         <f aca="false">SUM($I$9:I12)</f>
-        <v>46684.8480168067</v>
+        <v>46740.3102016807</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3475,11 +3475,11 @@
       </c>
       <c r="K13" s="39" t="n">
         <f aca="false">IF($I$15=0,0,I13/$I$15)</f>
-        <v>0.357576161267994</v>
+        <v>0.35735000277391</v>
       </c>
       <c r="L13" s="37" t="n">
         <f aca="false">SUM($I$9:I13)</f>
-        <v>78021.0543403361</v>
+        <v>78076.5165252101</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3521,11 +3521,11 @@
       </c>
       <c r="K14" s="39" t="n">
         <f aca="false">IF($I$15=0,0,I14/$I$15)</f>
-        <v>0.109704958505114</v>
+        <v>0.109635572704559</v>
       </c>
       <c r="L14" s="37" t="n">
         <f aca="false">SUM($I$9:I14)</f>
-        <v>87635.0543403361</v>
+        <v>87690.5165252101</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3548,19 +3548,19 @@
       </c>
       <c r="G15" s="41" t="n">
         <f aca="false">SUM(G9:G14)</f>
-        <v>79668.2312184874</v>
+        <v>79718.6513865546</v>
       </c>
       <c r="H15" s="41" t="n">
         <f aca="false">SUM(H9:H14)</f>
-        <v>7966.82312184874</v>
+        <v>7971.86513865546</v>
       </c>
       <c r="I15" s="41" t="n">
         <f aca="false">SUM(I9:I14)</f>
-        <v>87635.0543403361</v>
+        <v>87690.5165252101</v>
       </c>
       <c r="J15" s="42" t="n">
         <f aca="false">I15*Narxlar!$C$19</f>
-        <v>1042857146.65</v>
+        <v>1043517146.65</v>
       </c>
       <c r="K15" s="14" t="n">
         <f aca="false">SUM(K9:K14)</f>
@@ -4013,11 +4013,11 @@
       </c>
       <c r="C32" s="48" t="n">
         <f aca="false">$I$11*MAX(0,MIN($F$11,EOMONTH(C$29,0))-MAX($E$11,C$29)+1)/($F$11-$E$11+1)</f>
-        <v>2317.45913565426</v>
+        <v>2325.38230492197</v>
       </c>
       <c r="D32" s="48" t="n">
         <f aca="false">$I$11*MAX(0,MIN($F$11,EOMONTH(D$29,0))-MAX($E$11,D$29)+1)/($F$11-$E$11+1)</f>
-        <v>13904.7548139256</v>
+        <v>13952.2938295318</v>
       </c>
       <c r="E32" s="48" t="n">
         <f aca="false">$I$11*MAX(0,MIN($F$11,EOMONTH(E$29,0))-MAX($E$11,E$29)+1)/($F$11-$E$11+1)</f>
@@ -4106,11 +4106,11 @@
       </c>
       <c r="C36" s="41" t="n">
         <f aca="false">SUM(C30:C35)</f>
-        <v>14264.0599759904</v>
+        <v>14271.9831452581</v>
       </c>
       <c r="D36" s="41" t="n">
         <f aca="false">SUM(D30:D35)</f>
-        <v>49513.2642172869</v>
+        <v>49560.8032328932</v>
       </c>
       <c r="E36" s="41" t="n">
         <f aca="false">SUM(E30:E35)</f>
@@ -4127,11 +4127,11 @@
       </c>
       <c r="C37" s="42" t="n">
         <f aca="false">C36*Narxlar!$C$19</f>
-        <v>169742313.714286</v>
+        <v>169836599.428571</v>
       </c>
       <c r="D37" s="42" t="n">
         <f aca="false">D36*Narxlar!$C$19</f>
-        <v>589207844.185714</v>
+        <v>589773558.471429</v>
       </c>
       <c r="E37" s="42" t="n">
         <f aca="false">E36*Narxlar!$C$19</f>
@@ -5676,7 +5676,7 @@
       </c>
       <c r="D65" s="50" t="n">
         <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$345,'Hisob (batafsil)'!$K$5:$K$345,$A65)</f>
-        <v>4588.23529411765</v>
+        <v>4638.65546218487</v>
       </c>
       <c r="E65" s="51" t="n">
         <v>0</v>
@@ -5710,7 +5710,7 @@
       </c>
       <c r="N65" s="53" t="n">
         <f aca="false">$D65*G65</f>
-        <v>4588.23529411765</v>
+        <v>4638.65546218487</v>
       </c>
       <c r="O65" s="53" t="n">
         <f aca="false">$D65*H65</f>
@@ -8234,7 +8234,7 @@
       <c r="C107" s="11"/>
       <c r="D107" s="41" t="n">
         <f aca="false">SUM(D41:D106)</f>
-        <v>79668.2312184874</v>
+        <v>79718.6513865546</v>
       </c>
       <c r="E107" s="11"/>
       <c r="F107" s="11"/>
@@ -8253,7 +8253,7 @@
       </c>
       <c r="N107" s="41" t="n">
         <f aca="false">SUM(N41:N106)</f>
-        <v>14747.4672268908</v>
+        <v>14797.887394958</v>
       </c>
       <c r="O107" s="41" t="n">
         <f aca="false">SUM(O41:O106)</f>
@@ -10841,7 +10841,7 @@
       </c>
       <c r="T35" s="50" t="n">
         <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$345,'Hisob (batafsil)'!$B$5:$B$345,$A35,'Hisob (batafsil)'!$C$5:$C$345,"Konditsioner va ventilyatsiya")</f>
-        <v>17238.2352941176</v>
+        <v>17288.6554621849</v>
       </c>
       <c r="U35" s="50" t="n">
         <f aca="false">SUMIFS('Hisob (batafsil)'!$J$5:$J$345,'Hisob (batafsil)'!$B$5:$B$345,$A35,'Hisob (batafsil)'!$C$5:$C$345,"Mebel va interyer")</f>
@@ -10857,7 +10857,7 @@
       </c>
       <c r="X35" s="58" t="n">
         <f aca="false">C35+E35+G35+I35+K35+L35+M35+N35+O35+P35+Q35+R35+S35+T35+U35+V35+W35</f>
-        <v>24248.2016806723</v>
+        <v>24298.6218487395</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10938,7 +10938,7 @@
       </c>
       <c r="T36" s="41" t="n">
         <f aca="false">SUM(T28:T35)</f>
-        <v>17238.2352941176</v>
+        <v>17288.6554621849</v>
       </c>
       <c r="U36" s="41" t="n">
         <f aca="false">SUM(U28:U35)</f>
@@ -10954,7 +10954,7 @@
       </c>
       <c r="X36" s="41" t="n">
         <f aca="false">SUM(X28:X35)</f>
-        <v>36864.7016806723</v>
+        <v>36915.1218487395</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11354,7 +11354,7 @@
       </c>
       <c r="T43" s="62" t="n">
         <f aca="false">T7+T17+T25+T36+T41</f>
-        <v>18238.2352941176</v>
+        <v>18288.6554621849</v>
       </c>
       <c r="U43" s="62" t="n">
         <f aca="false">U7+U17+U25+U36+U41</f>
@@ -11370,7 +11370,7 @@
       </c>
       <c r="X43" s="62" t="n">
         <f aca="false">X7+X17+X25+X36+X41</f>
-        <v>79668.2312184874</v>
+        <v>79718.6513865546</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11402,7 +11402,7 @@
       <c r="W44" s="16"/>
       <c r="X44" s="64" t="n">
         <f aca="false">X43*Narxlar!$C$93</f>
-        <v>7966.82312184874</v>
+        <v>7971.86513865546</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11433,7 +11433,7 @@
       <c r="W45" s="20"/>
       <c r="X45" s="62" t="n">
         <f aca="false">X43+X44</f>
-        <v>87635.0543403361</v>
+        <v>87690.5165252101</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11464,7 +11464,7 @@
       <c r="W46" s="20"/>
       <c r="X46" s="22" t="n">
         <f aca="false">X45*Narxlar!$C$19</f>
-        <v>1042857146.65</v>
+        <v>1043517146.65</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12392,7 +12392,7 @@
         <v>344</v>
       </c>
       <c r="C55" s="66" t="n">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D55" s="6" t="s">
         <v>297</v>
@@ -23137,7 +23137,7 @@
       <c r="F311" s="74"/>
       <c r="G311" s="56" t="n">
         <f aca="false">Narxlar!$C$55</f>
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="H311" s="5" t="s">
         <v>297</v>
@@ -23148,7 +23148,7 @@
       </c>
       <c r="J311" s="76" t="n">
         <f aca="false">G311*I311</f>
-        <v>4588.23529411765</v>
+        <v>4638.65546218487</v>
       </c>
       <c r="K311" s="24" t="s">
         <v>142</v>
@@ -23302,7 +23302,7 @@
       <c r="I316" s="77"/>
       <c r="J316" s="12" t="n">
         <f aca="false">SUM(J294:J315)</f>
-        <v>24248.2016806723</v>
+        <v>24298.6218487395</v>
       </c>
     </row>
     <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24147,7 +24147,7 @@
       <c r="I346" s="77"/>
       <c r="J346" s="12" t="n">
         <f aca="false">J13+J27+J40+J54+J72+J87+J102+J118+J137+J155+J170+J185+J192+J219+J248+J256+J264+J282+J286+J291+J316+J325+J344</f>
-        <v>79668.2312184874</v>
+        <v>79718.6513865546</v>
       </c>
     </row>
   </sheetData>

</xml_diff>